<commit_message>
feat: enable config-validation by default and rename the sample to laser
- ship config-validation in default features; opt out with --no-default-features
- rename the sample ability, tags, code, and tests from fireball to laser
- drop the sample cooldown tag from blocked_tags so it no longer blocks recast
- remove fireball wording from the knowledge base and README
</commit_message>
<xml_diff>
--- a/config/tables/gas.tag.xlsx
+++ b/config/tables/gas.tag.xlsx
@@ -1,289 +1,195 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bevy\BevyProjects\bevy_gas\config\tables\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11775"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="11775" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tag" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>##var</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>##type</t>
-  </si>
-  <si>
-    <t>string!</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>##group</t>
-  </si>
-  <si>
-    <t>##</t>
-  </si>
-  <si>
-    <t>Stable gameplay tag name.</t>
-  </si>
-  <si>
-    <t>Designer description.</t>
-  </si>
-  <si>
-    <t>Ability</t>
-  </si>
-  <si>
-    <t>Root tag for abilities.</t>
-  </si>
-  <si>
-    <t>Ability.Fireball</t>
-  </si>
-  <si>
-    <t>Fireball ability identity.</t>
-  </si>
-  <si>
-    <t>Cooldown</t>
-  </si>
-  <si>
-    <t>Root tag for cooldown effects.</t>
-  </si>
-  <si>
-    <t>Cooldown.Fireball</t>
-  </si>
-  <si>
-    <t>Fireball cooldown is active.</t>
-  </si>
-  <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>Root tag for actor states.</t>
-  </si>
-  <si>
-    <t>State.Stunned</t>
-  </si>
-  <si>
-    <t>The actor cannot activate abilities.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="23">
     <font>
-      <sz val="11"/>
       <name val="Carlito"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Arial"/>
       <charset val="134"/>
-    </font>
-    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FF182238"/>
+    </font>
+    <font>
       <name val="Arial"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <color rgb="FF182238"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="36">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -601,175 +507,176 @@
     </border>
   </borders>
   <cellStyleXfs count="50">
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1016,7 +923,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -1025,7 +932,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -1038,11 +945,74 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1239,111 +1209,157 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="3" width="23" customWidth="1"/>
+    <col width="12" customWidth="1" style="7" min="1" max="1"/>
+    <col width="23" customWidth="1" style="7" min="2" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+    <row r="1" ht="30" customHeight="1" s="7">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>##var</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
       </c>
     </row>
-    <row r="2" ht="52" customHeight="1" spans="1:3">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
+    <row r="2" ht="52" customHeight="1" s="7">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>##type</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>string!</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1" spans="1:3">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+    <row r="3" ht="25" customHeight="1" s="7">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>##group</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
     </row>
-    <row r="4" ht="66" customHeight="1" spans="1:3">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
+    <row r="4" ht="66" customHeight="1" s="7">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>##</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Stable gameplay tag name.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Designer description.</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1" spans="1:3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>11</v>
+    <row r="5" ht="40" customHeight="1" s="7">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Ability</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Root tag for abilities.</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1" spans="1:3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>13</v>
+    <row r="6" ht="40" customHeight="1" s="7">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Ability.Laser</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Laser ability identity.</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1" spans="1:3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>15</v>
+    <row r="7" ht="40" customHeight="1" s="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Cooldown</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Root tag for cooldown effects.</t>
+        </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1" spans="1:3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>17</v>
+    <row r="8" ht="40" customHeight="1" s="7">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Cooldown.Laser</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Laser cooldown is active.</t>
+        </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1" spans="1:3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>19</v>
+    <row r="9" ht="40" customHeight="1" s="7">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Root tag for actor states.</t>
+        </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1" spans="1:3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>21</v>
+    <row r="10" ht="40" customHeight="1" s="7">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>State.Stunned</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>The actor cannot activate abilities.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>